<commit_message>
#8 BOM of changes updated
</commit_message>
<xml_diff>
--- a/Design-Files/Main-Board-V1.1/Deliverables/BOM/Client-BOM-Main-Board-V1.0.0.xlsx
+++ b/Design-Files/Main-Board-V1.1/Deliverables/BOM/Client-BOM-Main-Board-V1.0.0.xlsx
@@ -1,25 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\dominikschmidt-meditationdevice\Design-Files\Main-Board-V1.1\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C8460E-9A93-46D7-BF76-46C947953E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="354">
   <si>
     <t>#</t>
   </si>
@@ -126,9 +138,6 @@
     <t>C35</t>
   </si>
   <si>
-    <t>C36</t>
-  </si>
-  <si>
     <t>C42, C43</t>
   </si>
   <si>
@@ -180,9 +189,6 @@
     <t>LED1</t>
   </si>
   <si>
-    <t>LED2, LED3, LED4</t>
-  </si>
-  <si>
     <t>Q1</t>
   </si>
   <si>
@@ -198,9 +204,6 @@
     <t>R2, R28, R29, R38, R63, R68</t>
   </si>
   <si>
-    <t>R4, R20, R39</t>
-  </si>
-  <si>
     <t>R5, R15, R26, R30, R33</t>
   </si>
   <si>
@@ -231,9 +234,6 @@
     <t>R18</t>
   </si>
   <si>
-    <t>R19, R37, R41</t>
-  </si>
-  <si>
     <t>R23, R24</t>
   </si>
   <si>
@@ -714,12 +714,6 @@
     <t>PSPMAA0412-1R0M-ANP</t>
   </si>
   <si>
-    <t>XZVG68W-2</t>
-  </si>
-  <si>
-    <t>XZMDK68W-2</t>
-  </si>
-  <si>
     <t>AO3407</t>
   </si>
   <si>
@@ -1057,12 +1051,54 @@
   </si>
   <si>
     <t>IPS 2.1 inch 40PIN TFT LCD Capacitive Round Screen (Short Cable) ST7701S IC 480*480 SPI+RGB Interface HDMI-compatible Board</t>
+  </si>
+  <si>
+    <t>LED3, LED4</t>
+  </si>
+  <si>
+    <t>LED2</t>
+  </si>
+  <si>
+    <t>APHHS1005SURCK</t>
+  </si>
+  <si>
+    <t>Kingbright</t>
+  </si>
+  <si>
+    <t>APHHS1005CGCK</t>
+  </si>
+  <si>
+    <t>R4, R69</t>
+  </si>
+  <si>
+    <t>R20, R39</t>
+  </si>
+  <si>
+    <t>R37</t>
+  </si>
+  <si>
+    <t>R19, R41</t>
+  </si>
+  <si>
+    <t>C6, C36</t>
+  </si>
+  <si>
+    <t>R70</t>
+  </si>
+  <si>
+    <t>RES 49.9 OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>RC0603FR-0749R9L</t>
+  </si>
+  <si>
+    <t>49.9R</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1330,18 +1366,24 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>77</xdr:row>
+      <xdr:row>81</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>1295400</xdr:colOff>
-      <xdr:row>96</xdr:row>
+      <xdr:row>100</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1635,9 +1677,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1677,25 +1719,25 @@
         <v>21</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1711,19 +1753,19 @@
         <v>22</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="J3" s="7">
         <v>3</v>
@@ -1733,7 +1775,7 @@
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B74" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B78" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -1743,19 +1785,19 @@
         <v>23</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="J4" s="9">
         <v>7</v>
@@ -1775,19 +1817,19 @@
         <v>24</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
@@ -1807,19 +1849,19 @@
         <v>25</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1839,19 +1881,19 @@
         <v>26</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="J7" s="7">
         <v>3</v>
@@ -1871,19 +1913,19 @@
         <v>27</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1903,19 +1945,19 @@
         <v>28</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1935,19 +1977,19 @@
         <v>29</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="J10" s="9">
         <v>8</v>
@@ -1967,19 +2009,19 @@
         <v>30</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="J11" s="7">
         <v>11</v>
@@ -1999,19 +2041,19 @@
         <v>31</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="J12" s="9">
         <v>3</v>
@@ -2031,19 +2073,19 @@
         <v>32</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -2063,19 +2105,19 @@
         <v>33</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -2095,19 +2137,19 @@
         <v>34</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -2124,25 +2166,25 @@
         <v>2</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>35</v>
+        <v>349</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="J16" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16" s="9"/>
     </row>
@@ -2156,22 +2198,22 @@
         <v>2</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
@@ -2188,22 +2230,22 @@
         <v>6</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -2220,22 +2262,22 @@
         <v>3</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J19" s="7">
         <v>4</v>
@@ -2252,22 +2294,22 @@
         <v>4</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -2284,22 +2326,22 @@
         <v>5</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J21" s="7">
         <v>6</v>
@@ -2316,22 +2358,22 @@
         <v>6</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -2348,22 +2390,22 @@
         <v>6</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -2380,22 +2422,22 @@
         <v>7</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2412,22 +2454,22 @@
         <v>8</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2444,22 +2486,22 @@
         <v>9</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
@@ -2476,22 +2518,22 @@
         <v>8</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J27" s="7">
         <v>2</v>
@@ -2508,22 +2550,22 @@
         <v>10</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2540,22 +2582,22 @@
         <v>8</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2572,22 +2614,22 @@
         <v>11</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2604,22 +2646,22 @@
         <v>11</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -2636,22 +2678,22 @@
         <v>11</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2668,22 +2710,22 @@
         <v>12</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>231</v>
-      </c>
-      <c r="H33" s="7" t="s">
-        <v>285</v>
+        <v>344</v>
+      </c>
+      <c r="H33" s="9" t="s">
+        <v>343</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2700,283 +2742,279 @@
         <v>12</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>53</v>
+        <v>341</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>232</v>
+        <v>342</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>285</v>
+        <v>343</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J34" s="9">
+        <v>1</v>
+      </c>
+      <c r="K34" s="9"/>
+    </row>
+    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="1"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>340</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="F35" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>342</v>
+      </c>
+      <c r="H35" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>333</v>
+      </c>
+      <c r="J35" s="14">
         <v>3</v>
       </c>
-      <c r="K34" s="9"/>
-    </row>
-    <row r="35" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="1"/>
-      <c r="B35" s="11">
-        <f>ROW(B35) - ROW($B$2)</f>
-        <v>33</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>286</v>
-      </c>
-      <c r="I35" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="J35" s="7">
-        <v>1</v>
-      </c>
-      <c r="K35" s="7"/>
+      <c r="K35" s="16"/>
     </row>
     <row r="36" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B36) - ROW($B$2)</f>
         <v>34</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D36" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="G36" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>287</v>
+      <c r="D36" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>280</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="J36" s="9">
-        <v>2</v>
-      </c>
-      <c r="K36" s="9"/>
+        <v>333</v>
+      </c>
+      <c r="J36" s="7">
+        <v>1</v>
+      </c>
+      <c r="K36" s="7"/>
     </row>
     <row r="37" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
-        <f>ROW(B37) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="C37" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D37" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="G37" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>287</v>
+      <c r="D37" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="H37" s="9" t="s">
+        <v>281</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="J37" s="7">
-        <v>3</v>
-      </c>
-      <c r="K37" s="7"/>
-    </row>
-    <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>333</v>
+      </c>
+      <c r="J37" s="9">
+        <v>2</v>
+      </c>
+      <c r="K37" s="9"/>
+    </row>
+    <row r="38" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B38) - ROW($B$2)</f>
         <v>36</v>
       </c>
-      <c r="C38" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="G38" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="I38" s="10" t="s">
-        <v>316</v>
-      </c>
-      <c r="J38" s="9">
-        <v>2</v>
-      </c>
-      <c r="K38" s="9"/>
+      <c r="C38" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G38" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="J38" s="7">
+        <v>3</v>
+      </c>
+      <c r="K38" s="7"/>
     </row>
     <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
-        <f>ROW(B39) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="C39" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D39" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="G39" s="8" t="s">
-        <v>237</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="I39" s="8" t="s">
-        <v>317</v>
-      </c>
-      <c r="J39" s="7">
-        <v>6</v>
-      </c>
-      <c r="K39" s="7"/>
+      <c r="D39" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="H39" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="I39" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="J39" s="9">
+        <v>2</v>
+      </c>
+      <c r="K39" s="9"/>
     </row>
     <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B40) - ROW($B$2)</f>
         <v>38</v>
       </c>
       <c r="C40" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D40" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G40" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="H40" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="I40" s="10" t="s">
-        <v>318</v>
-      </c>
-      <c r="J40" s="9">
-        <v>3</v>
-      </c>
-      <c r="K40" s="9"/>
+      <c r="D40" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="I40" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="J40" s="7">
+        <v>6</v>
+      </c>
+      <c r="K40" s="7"/>
     </row>
     <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="11">
-        <f>ROW(B41) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>39</v>
       </c>
       <c r="C41" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D41" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="E41" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="G41" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="H41" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="I41" s="8" t="s">
-        <v>317</v>
-      </c>
-      <c r="J41" s="7">
-        <v>5</v>
-      </c>
-      <c r="K41" s="7"/>
+      <c r="D41" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="H41" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="I41" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="J41" s="9">
+        <v>2</v>
+      </c>
+      <c r="K41" s="9"/>
     </row>
     <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="11">
-        <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
+      <c r="B42" s="11"/>
       <c r="C42" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D42" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="G42" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="H42" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="I42" s="10" t="s">
-        <v>318</v>
-      </c>
-      <c r="J42" s="9">
-        <v>1</v>
-      </c>
-      <c r="K42" s="9"/>
+      <c r="D42" s="14" t="s">
+        <v>346</v>
+      </c>
+      <c r="E42" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="F42" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="G42" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="H42" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="I42" s="15" t="s">
+        <v>312</v>
+      </c>
+      <c r="J42" s="14">
+        <v>2</v>
+      </c>
+      <c r="K42" s="16" t="s">
+        <v>332</v>
+      </c>
     </row>
     <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
@@ -2987,32 +3025,30 @@
       <c r="C43" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D43" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="E43" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="F43" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="G43" s="15" t="s">
-        <v>239</v>
-      </c>
-      <c r="H43" s="14" t="s">
-        <v>271</v>
-      </c>
-      <c r="I43" s="15" t="s">
-        <v>319</v>
-      </c>
-      <c r="J43" s="14">
-        <v>3</v>
-      </c>
-      <c r="K43" s="16" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D43" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="G43" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="I43" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="J43" s="7">
+        <v>5</v>
+      </c>
+      <c r="K43" s="7"/>
+    </row>
+    <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
         <f t="shared" si="0"/>
@@ -3022,29 +3058,29 @@
         <v>14</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
       </c>
       <c r="K44" s="9"/>
     </row>
-    <row r="45" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="11">
         <f>ROW(B45) - ROW($B$2)</f>
@@ -3053,28 +3089,30 @@
       <c r="C45" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D45" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="E45" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="G45" s="8" t="s">
-        <v>242</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="I45" s="8" t="s">
-        <v>321</v>
-      </c>
-      <c r="J45" s="7">
-        <v>18</v>
-      </c>
-      <c r="K45" s="7"/>
+      <c r="D45" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E45" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="F45" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="G45" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="H45" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="I45" s="15" t="s">
+        <v>313</v>
+      </c>
+      <c r="J45" s="14">
+        <v>3</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>332</v>
+      </c>
     </row>
     <row r="46" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
@@ -3086,29 +3124,29 @@
         <v>14</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
       </c>
       <c r="K46" s="9"/>
     </row>
-    <row r="47" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="11">
         <f>ROW(B47) - ROW($B$2)</f>
@@ -3118,29 +3156,29 @@
         <v>14</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>289</v>
+        <v>265</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="J47" s="7">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="K47" s="7"/>
     </row>
-    <row r="48" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
         <f t="shared" si="0"/>
@@ -3150,57 +3188,57 @@
         <v>14</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>271</v>
+        <v>282</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
       </c>
       <c r="K48" s="9"/>
     </row>
-    <row r="49" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
         <f>ROW(B49) - ROW($B$2)</f>
         <v>47</v>
       </c>
-      <c r="C49" s="12" t="s">
+      <c r="C49" s="13" t="s">
         <v>14</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="J49" s="7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K49" s="7"/>
     </row>
@@ -3214,29 +3252,29 @@
         <v>14</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
       </c>
       <c r="K50" s="9"/>
     </row>
-    <row r="51" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="11">
         <f>ROW(B51) - ROW($B$2)</f>
@@ -3246,25 +3284,25 @@
         <v>14</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="J51" s="7">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K51" s="7"/>
     </row>
@@ -3278,25 +3316,25 @@
         <v>14</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J52" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K52" s="9"/>
     </row>
@@ -3310,22 +3348,22 @@
         <v>14</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>72</v>
+        <v>348</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="J53" s="7">
         <v>2</v>
@@ -3334,419 +3372,415 @@
     </row>
     <row r="54" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
-      <c r="B54" s="11">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-      <c r="C54" s="13" t="s">
+      <c r="B54" s="11"/>
+      <c r="C54" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D54" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="E54" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="F54" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G54" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="H54" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="I54" s="10" t="s">
-        <v>328</v>
-      </c>
-      <c r="J54" s="9">
-        <v>1</v>
-      </c>
-      <c r="K54" s="9"/>
+      <c r="D54" s="14" t="s">
+        <v>347</v>
+      </c>
+      <c r="E54" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F54" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="G54" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="H54" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="I54" s="15" t="s">
+        <v>320</v>
+      </c>
+      <c r="J54" s="14">
+        <v>1</v>
+      </c>
+      <c r="K54" s="16" t="s">
+        <v>332</v>
+      </c>
     </row>
     <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
-        <f>ROW(B55) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>53</v>
       </c>
       <c r="C55" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="E55" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="F55" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="G55" s="15" t="s">
-        <v>237</v>
-      </c>
-      <c r="H55" s="14" t="s">
-        <v>271</v>
-      </c>
-      <c r="I55" s="15" t="s">
-        <v>319</v>
-      </c>
-      <c r="J55" s="14">
-        <v>1</v>
-      </c>
-      <c r="K55" s="16" t="s">
-        <v>338</v>
-      </c>
+      <c r="D55" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="G55" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="H55" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="I55" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="J55" s="9">
+        <v>2</v>
+      </c>
+      <c r="K55" s="9"/>
     </row>
     <row r="56" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B56) - ROW($B$2)</f>
         <v>54</v>
       </c>
-      <c r="C56" s="13" t="s">
+      <c r="C56" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D56" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="E56" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="F56" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G56" s="10" t="s">
-        <v>252</v>
-      </c>
-      <c r="H56" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="I56" s="10" t="s">
-        <v>329</v>
-      </c>
-      <c r="J56" s="9">
-        <v>1</v>
-      </c>
-      <c r="K56" s="9"/>
+      <c r="D56" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="G56" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="H56" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="I56" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="J56" s="7">
+        <v>2</v>
+      </c>
+      <c r="K56" s="7"/>
     </row>
     <row r="57" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="11">
-        <f>ROW(B57) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>55</v>
       </c>
       <c r="C57" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D57" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E57" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="F57" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="G57" s="8" t="s">
-        <v>253</v>
-      </c>
-      <c r="H57" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="I57" s="8" t="s">
-        <v>330</v>
-      </c>
-      <c r="J57" s="7">
-        <v>1</v>
-      </c>
-      <c r="K57" s="7"/>
+      <c r="D57" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="G57" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="H57" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="I57" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="J57" s="9">
+        <v>1</v>
+      </c>
+      <c r="K57" s="9"/>
     </row>
     <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B58) - ROW($B$2)</f>
         <v>56</v>
       </c>
       <c r="C58" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D58" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="E58" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="F58" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G58" s="10" t="s">
-        <v>254</v>
-      </c>
-      <c r="H58" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="I58" s="10" t="s">
-        <v>331</v>
-      </c>
-      <c r="J58" s="9">
-        <v>1</v>
-      </c>
-      <c r="K58" s="9"/>
+      <c r="D58" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E58" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="F58" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="G58" s="15" t="s">
+        <v>231</v>
+      </c>
+      <c r="H58" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="I58" s="15" t="s">
+        <v>313</v>
+      </c>
+      <c r="J58" s="14">
+        <v>1</v>
+      </c>
+      <c r="K58" s="16" t="s">
+        <v>332</v>
+      </c>
     </row>
     <row r="59" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="11">
-        <f>ROW(B59) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>57</v>
       </c>
       <c r="C59" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D59" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="E59" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="F59" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="G59" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="H59" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="I59" s="8" t="s">
-        <v>332</v>
-      </c>
-      <c r="J59" s="7">
-        <v>1</v>
-      </c>
-      <c r="K59" s="7"/>
+      <c r="D59" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E59" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="G59" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="H59" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="I59" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="J59" s="9">
+        <v>1</v>
+      </c>
+      <c r="K59" s="9"/>
     </row>
     <row r="60" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B60) - ROW($B$2)</f>
         <v>58</v>
       </c>
       <c r="C60" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D60" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E60" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="F60" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G60" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="H60" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="I60" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="J60" s="9">
-        <v>1</v>
-      </c>
-      <c r="K60" s="9"/>
-    </row>
-    <row r="61" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D60" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="F60" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="G60" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="H60" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="I60" s="8" t="s">
+        <v>324</v>
+      </c>
+      <c r="J60" s="7">
+        <v>1</v>
+      </c>
+      <c r="K60" s="7"/>
+    </row>
+    <row r="61" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="11">
-        <f>ROW(B61) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="C61" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D61" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="E61" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="F61" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="G61" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="H61" s="7" t="s">
-        <v>290</v>
-      </c>
-      <c r="I61" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="J61" s="7">
-        <v>2</v>
-      </c>
-      <c r="K61" s="7"/>
-    </row>
-    <row r="62" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C61" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E61" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="F61" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="G61" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="H61" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="I61" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="J61" s="9">
+        <v>1</v>
+      </c>
+      <c r="K61" s="9"/>
+    </row>
+    <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B62) - ROW($B$2)</f>
         <v>60</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D62" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="E62" s="10" t="s">
-        <v>153</v>
+        <v>14</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E62" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="G62" s="10" t="s">
-        <v>190</v>
-      </c>
-      <c r="H62" s="9" t="s">
-        <v>291</v>
+        <v>183</v>
+      </c>
+      <c r="G62" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="H62" s="7" t="s">
+        <v>265</v>
       </c>
       <c r="I62" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="J62" s="9">
-        <v>3</v>
-      </c>
-      <c r="K62" s="9"/>
+        <v>326</v>
+      </c>
+      <c r="J62" s="7">
+        <v>1</v>
+      </c>
+      <c r="K62" s="7"/>
     </row>
     <row r="63" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="11">
-        <f>ROW(B63) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>61</v>
       </c>
-      <c r="C63" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D63" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="E63" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="F63" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="G63" s="8" t="s">
-        <v>191</v>
-      </c>
-      <c r="H63" s="7" t="s">
-        <v>292</v>
-      </c>
-      <c r="I63" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="J63" s="7">
-        <v>1</v>
-      </c>
-      <c r="K63" s="7"/>
+      <c r="C63" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D63" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E63" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="F63" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="G63" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="H63" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="I63" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="J63" s="9">
+        <v>1</v>
+      </c>
+      <c r="K63" s="9"/>
     </row>
     <row r="64" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
-      <c r="B64" s="11">
-        <f t="shared" si="0"/>
-        <v>62</v>
-      </c>
+      <c r="B64" s="11"/>
       <c r="C64" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D64" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E64" s="10" t="s">
-        <v>155</v>
+        <v>14</v>
+      </c>
+      <c r="D64" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>351</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="G64" s="10" t="s">
-        <v>257</v>
+        <v>182</v>
+      </c>
+      <c r="G64" s="8" t="s">
+        <v>352</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>293</v>
+        <v>265</v>
       </c>
       <c r="I64" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="J64" s="9">
-        <v>1</v>
-      </c>
-      <c r="K64" s="9"/>
-    </row>
-    <row r="65" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>353</v>
+      </c>
+      <c r="J64" s="7">
+        <v>1</v>
+      </c>
+      <c r="K64" s="7"/>
+    </row>
+    <row r="65" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="11">
         <f>ROW(B65) - ROW($B$2)</f>
         <v>63</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>193</v>
+        <v>334</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>258</v>
+        <v>185</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J65" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K65" s="7"/>
     </row>
-    <row r="66" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="11">
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="F66" s="9" t="s">
-        <v>194</v>
+        <v>149</v>
+      </c>
+      <c r="F66" s="7" t="s">
+        <v>334</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>259</v>
+        <v>186</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="I66" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J66" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K66" s="9"/>
     </row>
@@ -3757,32 +3791,32 @@
         <v>65</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>195</v>
+        <v>334</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>260</v>
+        <v>187</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J67" s="7">
         <v>1</v>
       </c>
       <c r="K67" s="7"/>
     </row>
-    <row r="68" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="11">
         <f t="shared" si="0"/>
@@ -3792,61 +3826,61 @@
         <v>18</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="I68" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J68" s="9">
         <v>1</v>
       </c>
       <c r="K68" s="9"/>
     </row>
-    <row r="69" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="11">
         <f>ROW(B69) - ROW($B$2)</f>
         <v>67</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="I69" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J69" s="7">
         <v>1</v>
       </c>
       <c r="K69" s="7"/>
     </row>
-    <row r="70" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1"/>
       <c r="B70" s="11">
         <f t="shared" si="0"/>
@@ -3856,22 +3890,22 @@
         <v>18</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="I70" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J70" s="9">
         <v>1</v>
@@ -3887,30 +3921,32 @@
       <c r="C71" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D71" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="E71" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="F71" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="G71" s="8" t="s">
-        <v>264</v>
-      </c>
-      <c r="H71" s="7" t="s">
-        <v>295</v>
-      </c>
-      <c r="I71" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="J71" s="7">
-        <v>1</v>
-      </c>
-      <c r="K71" s="7"/>
-    </row>
-    <row r="72" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D71" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="E71" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="F71" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="G71" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="H71" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="I71" s="15" t="s">
+        <v>313</v>
+      </c>
+      <c r="J71" s="14">
+        <v>1</v>
+      </c>
+      <c r="K71" s="16" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1"/>
       <c r="B72" s="11">
         <f t="shared" si="0"/>
@@ -3919,28 +3955,30 @@
       <c r="C72" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D72" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="E72" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="F72" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="G72" s="10" t="s">
-        <v>265</v>
-      </c>
-      <c r="H72" s="9" t="s">
-        <v>297</v>
-      </c>
-      <c r="I72" s="8" t="s">
-        <v>339</v>
-      </c>
-      <c r="J72" s="9">
-        <v>1</v>
-      </c>
-      <c r="K72" s="9"/>
+      <c r="D72" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="E72" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="F72" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="G72" s="15" t="s">
+        <v>255</v>
+      </c>
+      <c r="H72" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="I72" s="15" t="s">
+        <v>313</v>
+      </c>
+      <c r="J72" s="14">
+        <v>1</v>
+      </c>
+      <c r="K72" s="16" t="s">
+        <v>332</v>
+      </c>
     </row>
     <row r="73" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
@@ -3949,32 +3987,32 @@
         <v>71</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="G73" s="8" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J73" s="7">
         <v>1</v>
       </c>
       <c r="K73" s="7"/>
     </row>
-    <row r="74" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
       <c r="B74" s="11">
         <f t="shared" si="0"/>
@@ -3984,124 +4022,252 @@
         <v>18</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="F74" s="9" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="I74" s="8" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="J74" s="9">
         <v>1</v>
       </c>
       <c r="K74" s="9"/>
     </row>
-    <row r="75" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
       <c r="B75" s="11">
         <f>ROW(B75) - ROW($B$2)</f>
         <v>73</v>
       </c>
       <c r="C75" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D75" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E75" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="F75" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="G75" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="H75" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="I75" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="J75" s="7">
+        <v>1</v>
+      </c>
+      <c r="K75" s="7"/>
+    </row>
+    <row r="76" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="1"/>
+      <c r="B76" s="11">
+        <f t="shared" si="0"/>
+        <v>74</v>
+      </c>
+      <c r="C76" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E76" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="F76" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="G76" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="H76" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="I76" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="J76" s="9">
+        <v>1</v>
+      </c>
+      <c r="K76" s="9"/>
+    </row>
+    <row r="77" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="1"/>
+      <c r="B77" s="11">
+        <f>ROW(B77) - ROW($B$2)</f>
+        <v>75</v>
+      </c>
+      <c r="C77" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D77" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E77" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="F77" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="H77" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="I77" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="J77" s="7">
+        <v>1</v>
+      </c>
+      <c r="K77" s="7"/>
+    </row>
+    <row r="78" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="1"/>
+      <c r="B78" s="11">
+        <f t="shared" si="0"/>
+        <v>76</v>
+      </c>
+      <c r="C78" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D78" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E78" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="F78" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="G78" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="H78" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="I78" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="J78" s="9">
+        <v>1</v>
+      </c>
+      <c r="K78" s="9"/>
+    </row>
+    <row r="79" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="1"/>
+      <c r="B79" s="11">
+        <f>ROW(B79) - ROW($B$2)</f>
+        <v>77</v>
+      </c>
+      <c r="C79" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D75" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="E75" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="F75" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="G75" s="8" t="s">
-        <v>268</v>
-      </c>
-      <c r="H75" s="7" t="s">
-        <v>300</v>
-      </c>
-      <c r="I75" s="8" t="s">
+      <c r="D79" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E79" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="F79" s="7" t="s">
         <v>334</v>
       </c>
-      <c r="J75" s="7">
-        <v>1</v>
-      </c>
-      <c r="K75" s="7"/>
-    </row>
-    <row r="76" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="11">
-        <f t="shared" ref="B76:B77" si="1">ROW(B76) - ROW($B$2)</f>
-        <v>74</v>
-      </c>
-      <c r="C76" s="13" t="s">
-        <v>341</v>
-      </c>
-      <c r="D76" s="9" t="s">
+      <c r="G79" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="H79" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="I79" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="J79" s="7">
+        <v>1</v>
+      </c>
+      <c r="K79" s="7"/>
+    </row>
+    <row r="80" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B80" s="11">
+        <f t="shared" ref="B80:B81" si="1">ROW(B80) - ROW($B$2)</f>
+        <v>78</v>
+      </c>
+      <c r="C80" s="13" t="s">
+        <v>335</v>
+      </c>
+      <c r="D80" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="E80" s="10" t="s">
         <v>339</v>
       </c>
-      <c r="E76" s="10" t="s">
-        <v>345</v>
-      </c>
-      <c r="F76" s="9" t="s">
-        <v>339</v>
-      </c>
-      <c r="G76" s="10" t="s">
-        <v>341</v>
-      </c>
-      <c r="H76" s="9" t="s">
-        <v>339</v>
-      </c>
-      <c r="I76" s="10" t="s">
-        <v>339</v>
-      </c>
-      <c r="J76" s="9">
-        <v>1</v>
-      </c>
-      <c r="K76" s="17" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="11">
+      <c r="F80" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="G80" s="10" t="s">
+        <v>335</v>
+      </c>
+      <c r="H80" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="I80" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="J80" s="9">
+        <v>1</v>
+      </c>
+      <c r="K80" s="17" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="81" spans="2:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B81" s="11">
         <f t="shared" si="1"/>
-        <v>75</v>
-      </c>
-      <c r="C77" s="13" t="s">
-        <v>343</v>
-      </c>
-      <c r="D77" s="9" t="s">
-        <v>339</v>
-      </c>
-      <c r="E77" s="10" t="s">
-        <v>344</v>
-      </c>
-      <c r="F77" s="9" t="s">
-        <v>339</v>
-      </c>
-      <c r="G77" s="10" t="s">
-        <v>343</v>
-      </c>
-      <c r="H77" s="9" t="s">
-        <v>339</v>
-      </c>
-      <c r="I77" s="10" t="s">
-        <v>339</v>
-      </c>
-      <c r="J77" s="9">
-        <v>1</v>
-      </c>
-      <c r="K77" s="17" t="s">
-        <v>343</v>
+        <v>79</v>
+      </c>
+      <c r="C81" s="13" t="s">
+        <v>337</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="E81" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="F81" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="G81" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="H81" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="I81" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="J81" s="9">
+        <v>1</v>
+      </c>
+      <c r="K81" s="17" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -4109,8 +4275,8 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K77" r:id="rId1"/>
-    <hyperlink ref="K76" r:id="rId2"/>
+    <hyperlink ref="K81" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="K80" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>

</xml_diff>

<commit_message>
BOM diode D13 updated
</commit_message>
<xml_diff>
--- a/Design-Files/Main-Board-V1.1/Deliverables/BOM/Client-BOM-Main-Board-V1.0.0.xlsx
+++ b/Design-Files/Main-Board-V1.1/Deliverables/BOM/Client-BOM-Main-Board-V1.0.0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\dominikschmidt-meditationdevice\Design-Files\Main-Board-V1.1\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C8460E-9A93-46D7-BF76-46C947953E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7CAAB88-F298-4D79-86F0-151F4B92DED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -369,9 +369,6 @@
     <t>DIODE ZENER 3.3V 200MW SOD323F</t>
   </si>
   <si>
-    <t>DIODE GEN PURP 100V 300MA SOD123</t>
-  </si>
-  <si>
     <t>6V 2A 50A 1W -40℃~+85℃ 4A 4mΩ 5s 45mΩ 0805 Resettable Fuses ROHS</t>
   </si>
   <si>
@@ -693,9 +690,6 @@
     <t>MM3Z3V3B</t>
   </si>
   <si>
-    <t>1N4148W-7-F</t>
-  </si>
-  <si>
     <t>BSMD0805L-200</t>
   </si>
   <si>
@@ -1050,9 +1044,6 @@
     <t>3.7V 2000mAh 103450 Battery Lithium Polymer Batteries for POS Machines Bluetooth Speakers Anti-lost Devices Toys Camping Lights</t>
   </si>
   <si>
-    <t>IPS 2.1 inch 40PIN TFT LCD Capacitive Round Screen (Short Cable) ST7701S IC 480*480 SPI+RGB Interface HDMI-compatible Board</t>
-  </si>
-  <si>
     <t>LED3, LED4</t>
   </si>
   <si>
@@ -1093,6 +1084,15 @@
   </si>
   <si>
     <t>49.9R</t>
+  </si>
+  <si>
+    <t>IPS 2.1 inch 40PIN TFT LCD Capacitive Round Screen (Long Cable) ST7701S IC 480*480 SPI+RGB Interface HDMI-compatible Board</t>
+  </si>
+  <si>
+    <t>40V 1 Independent 450mV@1A 1A SOD-123 Schottky Diodes ROHS</t>
+  </si>
+  <si>
+    <t>1N5819HW-7-F</t>
   </si>
 </sst>
 </file>
@@ -1364,23 +1364,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>780723</xdr:colOff>
       <xdr:row>81</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>1295400</xdr:colOff>
-      <xdr:row>100</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>369846</xdr:colOff>
+      <xdr:row>110</xdr:row>
+      <xdr:rowOff>27742</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{749AA0B2-E6A2-DBD9-F99E-63EFC2D3D260}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1389,21 +1389,15 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4676775" y="21707475"/>
-          <a:ext cx="6648450" cy="3590925"/>
+          <a:off x="1599873" y="22555200"/>
+          <a:ext cx="10571448" cy="5409367"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1722,22 +1716,22 @@
         <v>91</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>329</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1756,16 +1750,16 @@
         <v>92</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="J3" s="7">
         <v>3</v>
@@ -1788,16 +1782,16 @@
         <v>93</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="J4" s="9">
         <v>7</v>
@@ -1820,16 +1814,16 @@
         <v>94</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
@@ -1852,16 +1846,16 @@
         <v>95</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1884,16 +1878,16 @@
         <v>96</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="J7" s="7">
         <v>3</v>
@@ -1916,16 +1910,16 @@
         <v>97</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1948,16 +1942,16 @@
         <v>98</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1980,16 +1974,16 @@
         <v>99</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="J10" s="9">
         <v>8</v>
@@ -2012,16 +2006,16 @@
         <v>100</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="J11" s="7">
         <v>11</v>
@@ -2044,16 +2038,16 @@
         <v>101</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="J12" s="9">
         <v>3</v>
@@ -2076,16 +2070,16 @@
         <v>102</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -2108,16 +2102,16 @@
         <v>103</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -2140,16 +2134,16 @@
         <v>104</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -2166,22 +2160,22 @@
         <v>2</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>105</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="J16" s="9">
         <v>2</v>
@@ -2204,16 +2198,16 @@
         <v>106</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
@@ -2236,16 +2230,16 @@
         <v>107</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -2268,16 +2262,16 @@
         <v>108</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J19" s="7">
         <v>4</v>
@@ -2300,16 +2294,16 @@
         <v>109</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -2332,16 +2326,16 @@
         <v>110</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J21" s="7">
         <v>6</v>
@@ -2364,23 +2358,23 @@
         <v>111</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -2393,19 +2387,19 @@
         <v>41</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>112</v>
+        <v>352</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>220</v>
+        <v>353</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -2425,19 +2419,19 @@
         <v>42</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2457,19 +2451,19 @@
         <v>43</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2489,19 +2483,19 @@
         <v>44</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
@@ -2521,19 +2515,19 @@
         <v>45</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J27" s="7">
         <v>2</v>
@@ -2553,19 +2547,19 @@
         <v>46</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2585,19 +2579,19 @@
         <v>47</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2617,19 +2611,19 @@
         <v>48</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2649,19 +2643,19 @@
         <v>49</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -2681,19 +2675,19 @@
         <v>50</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2713,19 +2707,19 @@
         <v>51</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2742,22 +2736,22 @@
         <v>12</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2771,22 +2765,22 @@
         <v>12</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="I35" s="15" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J35" s="14">
         <v>3</v>
@@ -2806,19 +2800,19 @@
         <v>52</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J36" s="7">
         <v>1</v>
@@ -2838,19 +2832,19 @@
         <v>53</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J37" s="9">
         <v>2</v>
@@ -2870,19 +2864,19 @@
         <v>54</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H38" s="7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="I38" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J38" s="7">
         <v>3</v>
@@ -2902,19 +2896,19 @@
         <v>55</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="J39" s="9">
         <v>2</v>
@@ -2934,19 +2928,19 @@
         <v>56</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H40" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I40" s="8" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="J40" s="7">
         <v>6</v>
@@ -2963,22 +2957,22 @@
         <v>14</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G41" s="10" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I41" s="10" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J41" s="9">
         <v>2</v>
@@ -2992,28 +2986,28 @@
         <v>14</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H42" s="14" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I42" s="15" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J42" s="14">
         <v>2</v>
       </c>
       <c r="K42" s="16" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3029,19 +3023,19 @@
         <v>57</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="J43" s="7">
         <v>5</v>
@@ -3061,19 +3055,19 @@
         <v>58</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
@@ -3093,25 +3087,25 @@
         <v>59</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G45" s="15" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H45" s="14" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I45" s="15" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="J45" s="14">
         <v>3</v>
       </c>
       <c r="K45" s="16" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3127,19 +3121,19 @@
         <v>60</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
@@ -3159,19 +3153,19 @@
         <v>61</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J47" s="7">
         <v>18</v>
@@ -3191,19 +3185,19 @@
         <v>62</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
@@ -3223,19 +3217,19 @@
         <v>63</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
@@ -3255,19 +3249,19 @@
         <v>64</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
@@ -3287,19 +3281,19 @@
         <v>65</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="J51" s="7">
         <v>10</v>
@@ -3319,19 +3313,19 @@
         <v>66</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J52" s="9">
         <v>1</v>
@@ -3348,22 +3342,22 @@
         <v>14</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J53" s="7">
         <v>2</v>
@@ -3377,28 +3371,28 @@
         <v>14</v>
       </c>
       <c r="D54" s="14" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F54" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G54" s="15" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H54" s="14" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I54" s="15" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J54" s="14">
         <v>1</v>
       </c>
       <c r="K54" s="16" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3414,19 +3408,19 @@
         <v>67</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G55" s="10" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I55" s="10" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J55" s="9">
         <v>2</v>
@@ -3446,19 +3440,19 @@
         <v>68</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="H56" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I56" s="8" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J56" s="7">
         <v>2</v>
@@ -3478,19 +3472,19 @@
         <v>69</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G57" s="10" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I57" s="10" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J57" s="9">
         <v>1</v>
@@ -3510,25 +3504,25 @@
         <v>70</v>
       </c>
       <c r="E58" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F58" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G58" s="15" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H58" s="14" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I58" s="15" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="J58" s="14">
         <v>1</v>
       </c>
       <c r="K58" s="16" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3544,19 +3538,19 @@
         <v>71</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F59" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G59" s="10" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I59" s="10" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J59" s="9">
         <v>1</v>
@@ -3576,19 +3570,19 @@
         <v>72</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G60" s="8" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="H60" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I60" s="8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J60" s="7">
         <v>1</v>
@@ -3608,19 +3602,19 @@
         <v>73</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G61" s="10" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I61" s="10" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J61" s="9">
         <v>1</v>
@@ -3640,19 +3634,19 @@
         <v>74</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G62" s="8" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="H62" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I62" s="8" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J62" s="7">
         <v>1</v>
@@ -3672,19 +3666,19 @@
         <v>75</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G63" s="10" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I63" s="10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J63" s="9">
         <v>1</v>
@@ -3698,22 +3692,22 @@
         <v>14</v>
       </c>
       <c r="D64" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>348</v>
+      </c>
+      <c r="F64" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="G64" s="8" t="s">
+        <v>349</v>
+      </c>
+      <c r="H64" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="I64" s="8" t="s">
         <v>350</v>
-      </c>
-      <c r="E64" s="8" t="s">
-        <v>351</v>
-      </c>
-      <c r="F64" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="G64" s="8" t="s">
-        <v>352</v>
-      </c>
-      <c r="H64" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="I64" s="8" t="s">
-        <v>353</v>
       </c>
       <c r="J64" s="7">
         <v>1</v>
@@ -3733,19 +3727,19 @@
         <v>76</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J65" s="7">
         <v>2</v>
@@ -3765,19 +3759,19 @@
         <v>77</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="I66" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J66" s="9">
         <v>3</v>
@@ -3797,19 +3791,19 @@
         <v>78</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J67" s="7">
         <v>1</v>
@@ -3829,19 +3823,19 @@
         <v>79</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="I68" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J68" s="9">
         <v>1</v>
@@ -3861,19 +3855,19 @@
         <v>80</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="I69" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J69" s="7">
         <v>1</v>
@@ -3893,19 +3887,19 @@
         <v>81</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="I70" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J70" s="9">
         <v>1</v>
@@ -3925,25 +3919,25 @@
         <v>82</v>
       </c>
       <c r="E71" s="15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F71" s="14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G71" s="15" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="H71" s="14" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="I71" s="15" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="J71" s="14">
         <v>1</v>
       </c>
       <c r="K71" s="16" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="72" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3959,25 +3953,25 @@
         <v>83</v>
       </c>
       <c r="E72" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F72" s="14" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G72" s="15" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H72" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="I72" s="15" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="J72" s="14">
         <v>1</v>
       </c>
       <c r="K72" s="16" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="73" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3993,19 +3987,19 @@
         <v>84</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G73" s="8" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J73" s="7">
         <v>1</v>
@@ -4025,19 +4019,19 @@
         <v>85</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F74" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="I74" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J74" s="9">
         <v>1</v>
@@ -4057,19 +4051,19 @@
         <v>86</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G75" s="8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H75" s="7" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I75" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J75" s="7">
         <v>1</v>
@@ -4089,19 +4083,19 @@
         <v>87</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F76" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G76" s="10" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="I76" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J76" s="9">
         <v>1</v>
@@ -4121,19 +4115,19 @@
         <v>88</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G77" s="8" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H77" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I77" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J77" s="7">
         <v>1</v>
@@ -4153,19 +4147,19 @@
         <v>89</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F78" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G78" s="10" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="H78" s="9" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="I78" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J78" s="9">
         <v>1</v>
@@ -4185,19 +4179,19 @@
         <v>90</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G79" s="8" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H79" s="7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="I79" s="8" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J79" s="7">
         <v>1</v>
@@ -4210,31 +4204,31 @@
         <v>78</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D80" s="9" t="s">
+        <v>331</v>
+      </c>
+      <c r="E80" s="10" t="s">
+        <v>351</v>
+      </c>
+      <c r="F80" s="9" t="s">
+        <v>331</v>
+      </c>
+      <c r="G80" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="E80" s="10" t="s">
-        <v>339</v>
-      </c>
-      <c r="F80" s="9" t="s">
-        <v>333</v>
-      </c>
-      <c r="G80" s="10" t="s">
-        <v>335</v>
-      </c>
       <c r="H80" s="9" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="I80" s="10" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J80" s="9">
         <v>1</v>
       </c>
       <c r="K80" s="17" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="81" spans="2:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4243,31 +4237,31 @@
         <v>79</v>
       </c>
       <c r="C81" s="13" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F81" s="9" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="G81" s="10" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="H81" s="9" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="I81" s="10" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J81" s="9">
         <v>1</v>
       </c>
       <c r="K81" s="17" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>